<commit_message>
feat(templates): expand AliExpress, eBay, and Wish after-sales scripts
Add 15 high-intent marketplace case templates and refresh the index, README, and offline packs to 1,480.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/dist/customer-service-scripts.xlsx
+++ b/dist/customer-service-scripts.xlsx
@@ -768,7 +768,7 @@
         <v>AliExpress-售后</v>
       </c>
       <c r="E13">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F13" t="str">
         <v>platforms/aliexpress/aftersales.md</v>
@@ -906,7 +906,7 @@
         <v>eBay-售后</v>
       </c>
       <c r="E19">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F19" t="str">
         <v>platforms/ebay/aftersales.md</v>
@@ -1320,7 +1320,7 @@
         <v>Wish-售后</v>
       </c>
       <c r="E37">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F37" t="str">
         <v>platforms/wish/aftersales.md</v>
@@ -3197,7 +3197,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G16"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -3561,9 +3561,160 @@
         <v>AliExpress · 售后</v>
       </c>
     </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>物流延误安抚</v>
+      </c>
+      <c r="C12" t="str">
+        <v>跨境物流超时，但包裹仍有轨迹、买家准备开纠纷</v>
+      </c>
+      <c r="D12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! I checked order #[Order Number] and the package is still moving.
+Tracking: [Tracking Number]
+Carrier: [Carrier]
+Latest status: [Status]
+Last location: [Location]
+New estimated delivery: [New ETA]
+International transit can take longer at customs or the last-mile depot. I have also extended buyer protection until [Protection End Date].
+If there is no new scan by [Follow-up Date], we can offer:
+1) Keep waiting with protection extended
+2) Full refund now
+3) Resend if stock is available
+Which option do you prefer?</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Order Number、Tracking Number、Carrier、Status、Location、New ETA、Protection End Date、Follow-up Date</v>
+      </c>
+      <c r="F12" t="str">
+        <v>platforms/aliexpress/aftersales.md</v>
+      </c>
+      <c r="G12" t="str">
+        <v>AliExpress · 售后</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>纠纷举证引导</v>
+      </c>
+      <c r="C13" t="str">
+        <v>买家已开纠纷，需要双方补充照片、物流和沟通记录</v>
+      </c>
+      <c r="D13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! To resolve the dispute for order #[Order Number] faster, please upload these items in the AliExpress dispute:
+1) Photos or video of the issue
+2) Photo of the product label or SKU
+3) Photo of the outer package and shipping label
+4) Your preferred solution
+I will also upload:
+• Shipping proof and tracking
+• Pre-shipment quality photos
+• Our previous message records
+Once both sides submit evidence, I can offer a fair proposal within [Time]. Please keep the dispute open so we can settle it inside AliExpress.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Order Number、Time</v>
+      </c>
+      <c r="F13" t="str">
+        <v>platforms/aliexpress/aftersales.md</v>
+      </c>
+      <c r="G13" t="str">
+        <v>AliExpress · 售后</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>国际退货部分退款</v>
+      </c>
+      <c r="C14" t="str">
+        <v>退货运费高于商品价值，协商买家留货并接受部分退款</v>
+      </c>
+      <c r="D14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! I understand you want a refund for order #[Order Number].
+Because international return shipping can cost more than the item, I recommend a keep-the-item solution:
+• Partial refund: $[Amount] ([X]%)
+• Plus coupon: $[Coupon Amount] for your next order
+• No return shipping needed
+Alternative: full refund after you return the item. Return shipping is usually the buyer's responsibility unless the item is defective or wrong.
+If this works, please accept the proposal in the dispute and I will process it right away.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Order Number、Amount、X、Coupon Amount</v>
+      </c>
+      <c r="F14" t="str">
+        <v>platforms/aliexpress/aftersales.md</v>
+      </c>
+      <c r="G14" t="str">
+        <v>AliExpress · 售后</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>保护期延长说明</v>
+      </c>
+      <c r="C15" t="str">
+        <v>买家担心 AliExpress 买家保护即将到期</v>
+      </c>
+      <c r="D15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! Buyer protection for order #[Order Number] is still active.
+Current protection end date: [Protection End Date]
+Tracking status: [Status]
+I have requested an extension so you stay covered while we wait for delivery or review your case. You do not need to open a dispute yet unless you prefer to start one now.
+If the package still has not arrived by [Follow-up Date], message me and I will help with refund or replacement under AliExpress Buyer Protection.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Order Number、Protection End Date、Status、Follow-up Date</v>
+      </c>
+      <c r="F15" t="str">
+        <v>platforms/aliexpress/aftersales.md</v>
+      </c>
+      <c r="G15" t="str">
+        <v>AliExpress · 售后</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>平台介入降级</v>
+      </c>
+      <c r="C16" t="str">
+        <v>纠纷已升级平台介入，卖家提出可接受方案避免恶化</v>
+      </c>
+      <c r="D16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! I see AliExpress has been asked to step in on order #[Order Number].
+I still want to settle this with you directly. My updated offer:
+• Resolution: [Resolution Option]
+• Amount: $[Amount]
+• Extra apology coupon: $[Coupon Amount]
+Please review the proposal in the dispute. If you accept, AliExpress can close the case faster and you will not need to wait for a platform decision.
+If you need a different option, tell me what would feel fair and I will adjust the proposal.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Order Number、Resolution Option、Amount、Coupon Amount</v>
+      </c>
+      <c r="F16" t="str">
+        <v>platforms/aliexpress/aftersales.md</v>
+      </c>
+      <c r="G16" t="str">
+        <v>AliExpress · 售后</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5477,7 +5628,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G16"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -5741,9 +5892,155 @@
         <v>eBay · 售后</v>
       </c>
     </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>INR 未收到货 Case</v>
+      </c>
+      <c r="C12" t="str">
+        <v>买家开启 Item Not Received case，需要核对物流并给出时限</v>
+      </c>
+      <c r="D12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! I'm sorry you have not received order #[Order Number].
+I checked the eBay tracking:
+• Tracking number: [Tracking Number]
+• Carrier: [Carrier]
+• Latest status: [Status]
+• Last scan: [Latest Scan]
+Please allow until [Follow-up Date] for final delivery. If it still does not arrive, I will close this under eBay Money Back Guarantee with a full refund of $[Amount] or send a replacement if stock is available.
+Please keep the case on eBay so the refund can be processed through official channels.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Order Number、Tracking Number、Carrier、Status、Latest Scan、Follow-up Date、Amount</v>
+      </c>
+      <c r="F12" t="str">
+        <v>platforms/ebay/aftersales.md</v>
+      </c>
+      <c r="G12" t="str">
+        <v>eBay · 售后</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>退货标签无法使用</v>
+      </c>
+      <c r="C13" t="str">
+        <v>买家申请退货后，eBay 退货标签无法打印或承运商拒收</v>
+      </c>
+      <c r="D13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! Sorry the return label is not working for order #[Order Number].
+Please try:
+1) Open the return from Purchase History
+2) Download the latest eBay return label
+3) Take the package to [Drop Off Location]
+If it still fails, send me a screenshot of the error. I can request a new label or approve another return method before [Return Deadline].
+Once the item is scanned, I will process the refund of $[Amount] within [Time] business days after we receive it.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Order Number、Drop Off Location、Return Deadline、Amount、Time</v>
+      </c>
+      <c r="F13" t="str">
+        <v>platforms/ebay/aftersales.md</v>
+      </c>
+      <c r="G13" t="str">
+        <v>eBay · 售后</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Case 降级协商</v>
+      </c>
+      <c r="C14" t="str">
+        <v>买家已开 eBay case，卖家希望在平台裁决前达成协议</v>
+      </c>
+      <c r="D14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! I see a case is open for order #[Order Number]. I want to resolve this before it needs more eBay review.
+Please confirm the issue: [Issue].
+I can offer one of these options now:
+1) Full refund after return
+2) Partial refund of $[Amount] and you keep the item
+3) Replacement shipped with tracking
+Reply with your preferred option in eBay Messages. If you accept, please also accept the offer in the case so it can be closed cleanly.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Order Number、Issue、Amount</v>
+      </c>
+      <c r="F14" t="str">
+        <v>platforms/ebay/aftersales.md</v>
+      </c>
+      <c r="G14" t="str">
+        <v>eBay · 售后</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>SNAD 照片核验</v>
+      </c>
+      <c r="C15" t="str">
+        <v>买家以 Significantly Not As Described 申请退货，需要证据后再处理</v>
+      </c>
+      <c r="D15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! I'm sorry the item from order #[Order Number] did not match the listing.
+To review the SNAD claim, please send photos of:
+1) The item you received
+2) Any defect or difference from the listing
+3) The packing and shipping label
+After I review the photos, I can offer a return with prepaid label, a partial refund of $[Amount], or a replacement if available.
+Thank you for giving me the chance to make this right inside eBay.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Order Number、Amount</v>
+      </c>
+      <c r="F15" t="str">
+        <v>platforms/ebay/aftersales.md</v>
+      </c>
+      <c r="G15" t="str">
+        <v>eBay · 售后</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Money Back Guarantee 时限说明</v>
+      </c>
+      <c r="C16" t="str">
+        <v>买家询问 eBay 退款保障何时到账、还要等多久</v>
+      </c>
+      <c r="D16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hello! Your case for order #[Order Number] is covered by eBay Money Back Guarantee.
+Current status: [Case Status]
+Approved amount: $[Amount]
+Refund method: [Payment Method]
+Expected posting time: [Time]
+eBay or PayPal has to release the refund to your original payment method. If it does not appear by [Follow-up Date], send me a screenshot and I will help you check the case timeline.
+All refunds will stay on official eBay or PayPal channels.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Order Number、Case Status、Amount、Payment Method、Time、Follow-up Date</v>
+      </c>
+      <c r="F16" t="str">
+        <v>platforms/ebay/aftersales.md</v>
+      </c>
+      <c r="G16" t="str">
+        <v>eBay · 售后</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -13692,7 +13989,7 @@
 
 <file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G16"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -14021,9 +14318,158 @@
         <v>Wish · 售后</v>
       </c>
     </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>超长物流安抚</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Wish 标准物流远超预计时效，买家担心包裹丢失</v>
+      </c>
+      <c r="D12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Sorry the delivery is taking longer than expected! 😢
+Order: [Order Number]
+Tracking: [Tracking Number]
+Latest status: [Status]
+New estimated delivery: [New ETA]
+Wish standard shipping can take extra time in transit or customs. You're still covered by Wish buyer protection until [Protection End Date].
+If there is no new update by [Follow-up Date], we can:
+• Issue a full refund
+• Send a replacement if stock is available
+Hang tight - we'll make it right! 🛡️</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Order Number、Tracking Number、Status、New ETA、Protection End Date、Follow-up Date</v>
+      </c>
+      <c r="F12" t="str">
+        <v>platforms/wish/aftersales.md</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Wish · 售后</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>低价商品免退货退款</v>
+      </c>
+      <c r="C13" t="str">
+        <v>商品单价低、退货不划算，直接退款或补发</v>
+      </c>
+      <c r="D13" t="str" xml:space="preserve">
+        <v xml:space="preserve">We're sorry about the issue with [Product Name]! 😔
+Because return shipping can cost more than the item, you do not need to send it back.
+Please choose:
+1) Full refund of $[Amount]
+2) Free replacement if stock is available
+3) Partial refund of $[Amount] and keep the item
+Reply with your choice and we'll process it in the Wish app. 💙</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Product Name、Amount</v>
+      </c>
+      <c r="F13" t="str">
+        <v>platforms/wish/aftersales.md</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Wish · 售后</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>无轨迹包裹核查</v>
+      </c>
+      <c r="C14" t="str">
+        <v>订单已发货但长期没有有效物流轨迹</v>
+      </c>
+      <c r="D14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Thanks for waiting! I checked order [Order Number] and tracking is not updating yet.
+Carrier: [Carrier]
+Tracking number: [Tracking Number]
+Ship date: [Date]
+Sometimes Wish economy shipping updates late. If there is still no scan by [Follow-up Date], we will treat it as lost and help you get a refund or replacement under Wish protection.
+Please confirm your shipping address is still [Shipping Address]. 📦</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Order Number、Carrier、Tracking Number、Date、Follow-up Date、Shipping Address</v>
+      </c>
+      <c r="F14" t="str">
+        <v>platforms/wish/aftersales.md</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Wish · 售后</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>买家保护申请引导</v>
+      </c>
+      <c r="C15" t="str">
+        <v>买家要申请 Wish Refund/Buyer Protection，需要正确提交材料</v>
+      </c>
+      <c r="D15" t="str" xml:space="preserve">
+        <v xml:space="preserve">You can use Wish buyer protection for this order. 🛡️
+Please open:
+Wish app → Order History → [Order Number] → Request Refund / Help
+Upload:
+1) Photos of the issue
+2) A short video if it is a function problem
+3) The reason: [Issue]
+We will review it quickly. If approved, refund or replacement can be processed without extra back-and-forth.
+Need help tapping the right button? Send a screenshot and we'll guide you! 💬</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Order Number、Issue</v>
+      </c>
+      <c r="F15" t="str">
+        <v>platforms/wish/aftersales.md</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Wish · 售后</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>售后优惠补偿</v>
+      </c>
+      <c r="C16" t="str">
+        <v>问题已解决后，用优惠券或折扣鼓励复购</v>
+      </c>
+      <c r="D16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Thank you for giving us a chance to fix this! 💜
+As an apology, we added:
+• Coupon: [Coupon Amount]
+• Valid until: [Date]
+• Eligible items: [Eligible Items]
+You can find it in your Wish account coupons. If anything still feels unresolved, message us before your next order and we'll help first.
+We appreciate your patience! ✨</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Coupon Amount、Date、Eligible Items</v>
+      </c>
+      <c r="F16" t="str">
+        <v>platforms/wish/aftersales.md</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Wish · 售后</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>